<commit_message>
Fix column detection: never map اسم المديرية/المركز to patient name
The header auto-detection matched the bare word اسم, so a column like
اسم المديرية (directorate) was grabbed as the patient name before reaching
اسم المراجع. Reworked mapping to use strong, specific keywords per field
(with the patient name requiring مراجع/مريض/مستفيد or a guarded الاسم
fallback that excludes directorate/center/etc.), assign each column once,
and normalize ة/ى/diacritics. Added a regression test suite and updated the
sample generator to mirror a real MOH export (directorate + center columns
before the name).

Co-authored-by: buddizzz <buddizzz@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/samples/family-medicine.xlsx
+++ b/samples/family-medicine.xlsx
@@ -397,149 +397,185 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:I6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>اسم المديرية</v>
+      </c>
+      <c r="B1" t="str">
+        <v>اسم المركز الصحي</v>
+      </c>
+      <c r="C1" t="str">
         <v>اسم المراجع</v>
       </c>
-      <c r="B1" t="str">
+      <c r="D1" t="str">
         <v>رقم الهوية</v>
       </c>
-      <c r="C1" t="str">
+      <c r="E1" t="str">
         <v>موعد الحجز</v>
       </c>
-      <c r="D1" t="str">
+      <c r="F1" t="str">
         <v>وقت الحجز</v>
       </c>
-      <c r="E1" t="str">
+      <c r="G1" t="str">
         <v>اسم الطبيب</v>
       </c>
-      <c r="F1" t="str">
+      <c r="H1" t="str">
         <v>اسم التخصص</v>
       </c>
-      <c r="G1" t="str">
-        <v>رقم الاتصال</v>
+      <c r="I1" t="str">
+        <v>رقم الجوال</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
+        <v>مديرية الشؤون الصحية بالرياض</v>
+      </c>
+      <c r="B2" t="str">
+        <v>مركز صحي النخيل</v>
+      </c>
+      <c r="C2" t="str">
         <v>محمد أحمد الغامدي</v>
       </c>
-      <c r="B2" t="str">
+      <c r="D2" t="str">
         <v>1012345678</v>
       </c>
-      <c r="C2" t="str">
+      <c r="E2" t="str">
         <v>2026-08-12</v>
       </c>
-      <c r="D2" t="str">
+      <c r="F2" t="str">
         <v>09:00</v>
       </c>
-      <c r="E2" t="str">
+      <c r="G2" t="str">
         <v>د. سعاد المطيري</v>
       </c>
-      <c r="F2" t="str">
+      <c r="H2" t="str">
         <v>طب الأسرة</v>
       </c>
-      <c r="G2" t="str">
+      <c r="I2" t="str">
         <v>0501234567</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
+        <v>مديرية الشؤون الصحية بالرياض</v>
+      </c>
+      <c r="B3" t="str">
+        <v>مركز صحي النخيل</v>
+      </c>
+      <c r="C3" t="str">
         <v>نورة سعد القحطاني</v>
       </c>
-      <c r="B3" t="str">
+      <c r="D3" t="str">
         <v>1023456789</v>
       </c>
-      <c r="C3" t="str">
+      <c r="E3" t="str">
         <v>2026-08-12</v>
       </c>
-      <c r="D3" t="str">
+      <c r="F3" t="str">
         <v>09:30</v>
       </c>
-      <c r="E3" t="str">
+      <c r="G3" t="str">
         <v>د. خالد العتيبي</v>
       </c>
-      <c r="F3" t="str">
+      <c r="H3" t="str">
         <v>طب الأسرة</v>
       </c>
-      <c r="G3" t="str">
+      <c r="I3" t="str">
         <v>0552345678</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
+        <v>مديرية الشؤون الصحية بالرياض</v>
+      </c>
+      <c r="B4" t="str">
+        <v>مركز صحي العليا</v>
+      </c>
+      <c r="C4" t="str">
         <v>عبدالله فهد الشهري</v>
       </c>
-      <c r="B4" t="str">
+      <c r="D4" t="str">
         <v>1034567890</v>
       </c>
-      <c r="C4" t="str">
+      <c r="E4" t="str">
         <v>2026-08-12</v>
       </c>
-      <c r="D4" t="str">
+      <c r="F4" t="str">
         <v>10:00</v>
       </c>
-      <c r="E4" t="str">
+      <c r="G4" t="str">
         <v>د. سعاد المطيري</v>
       </c>
-      <c r="F4" t="str">
+      <c r="H4" t="str">
         <v>طب الأسرة</v>
       </c>
-      <c r="G4" t="str">
+      <c r="I4" t="str">
         <v>0533456789</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
+        <v>مديرية الشؤون الصحية بالرياض</v>
+      </c>
+      <c r="B5" t="str">
+        <v>مركز صحي العليا</v>
+      </c>
+      <c r="C5" t="str">
         <v>ريم ناصر الدوسري</v>
       </c>
-      <c r="B5" t="str">
+      <c r="D5" t="str">
         <v>1045678901</v>
       </c>
-      <c r="C5" t="str">
+      <c r="E5" t="str">
         <v>2026-08-13</v>
       </c>
-      <c r="D5" t="str">
+      <c r="F5" t="str">
         <v>10:30</v>
       </c>
-      <c r="E5" t="str">
+      <c r="G5" t="str">
         <v>د. خالد العتيبي</v>
       </c>
-      <c r="F5" t="str">
+      <c r="H5" t="str">
         <v>طب الأسرة</v>
       </c>
-      <c r="G5" t="str">
+      <c r="I5" t="str">
         <v>0544567890</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
+        <v>مديرية الشؤون الصحية بالرياض</v>
+      </c>
+      <c r="B6" t="str">
+        <v>مركز صحي الملز</v>
+      </c>
+      <c r="C6" t="str">
         <v>سلطان عمر الحربي</v>
       </c>
-      <c r="B6" t="str">
+      <c r="D6" t="str">
         <v>1056789012</v>
       </c>
-      <c r="C6" t="str">
+      <c r="E6" t="str">
         <v>2026-08-13</v>
       </c>
-      <c r="D6" t="str">
+      <c r="F6" t="str">
         <v>11:00</v>
       </c>
-      <c r="E6" t="str">
+      <c r="G6" t="str">
         <v>د. منى الزهراني</v>
       </c>
-      <c r="F6" t="str">
+      <c r="H6" t="str">
         <v>طب الأسرة</v>
       </c>
-      <c r="G6" t="str">
+      <c r="I6" t="str">
         <v>0565678901</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Show appointment start time and patient arrival date on cards
Map Excel "وقت بداية الموعد" and "تاريخ وصول المراجع" into patient
records, update the card labels, and keep legacy "وقت الحجز" working.

Co-authored-by: buddizzz <buddizzz@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/samples/family-medicine.xlsx
+++ b/samples/family-medicine.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:J6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -416,15 +416,18 @@
         <v>موعد الحجز</v>
       </c>
       <c r="F1" t="str">
-        <v>وقت الحجز</v>
+        <v>وقت بداية الموعد</v>
       </c>
       <c r="G1" t="str">
+        <v>تاريخ وصول المراجع</v>
+      </c>
+      <c r="H1" t="str">
         <v>اسم الطبيب</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>اسم التخصص</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>رقم الجوال</v>
       </c>
     </row>
@@ -448,12 +451,15 @@
         <v>09:00</v>
       </c>
       <c r="G2" t="str">
+        <v>2026-08-12</v>
+      </c>
+      <c r="H2" t="str">
         <v>د. سعاد المطيري</v>
       </c>
-      <c r="H2" t="str">
+      <c r="I2" t="str">
         <v>طب الأسرة</v>
       </c>
-      <c r="I2" t="str">
+      <c r="J2" t="str">
         <v>0501234567</v>
       </c>
     </row>
@@ -477,12 +483,15 @@
         <v>09:30</v>
       </c>
       <c r="G3" t="str">
+        <v>2026-08-12</v>
+      </c>
+      <c r="H3" t="str">
         <v>د. خالد العتيبي</v>
       </c>
-      <c r="H3" t="str">
+      <c r="I3" t="str">
         <v>طب الأسرة</v>
       </c>
-      <c r="I3" t="str">
+      <c r="J3" t="str">
         <v>0552345678</v>
       </c>
     </row>
@@ -506,12 +515,15 @@
         <v>10:00</v>
       </c>
       <c r="G4" t="str">
+        <v>2026-08-12</v>
+      </c>
+      <c r="H4" t="str">
         <v>د. سعاد المطيري</v>
       </c>
-      <c r="H4" t="str">
+      <c r="I4" t="str">
         <v>طب الأسرة</v>
       </c>
-      <c r="I4" t="str">
+      <c r="J4" t="str">
         <v>0533456789</v>
       </c>
     </row>
@@ -535,12 +547,15 @@
         <v>10:30</v>
       </c>
       <c r="G5" t="str">
+        <v>2026-08-13</v>
+      </c>
+      <c r="H5" t="str">
         <v>د. خالد العتيبي</v>
       </c>
-      <c r="H5" t="str">
+      <c r="I5" t="str">
         <v>طب الأسرة</v>
       </c>
-      <c r="I5" t="str">
+      <c r="J5" t="str">
         <v>0544567890</v>
       </c>
     </row>
@@ -564,18 +579,21 @@
         <v>11:00</v>
       </c>
       <c r="G6" t="str">
+        <v>2026-08-13</v>
+      </c>
+      <c r="H6" t="str">
         <v>د. منى الزهراني</v>
       </c>
-      <c r="H6" t="str">
+      <c r="I6" t="str">
         <v>طب الأسرة</v>
       </c>
-      <c r="I6" t="str">
+      <c r="J6" t="str">
         <v>0565678901</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>